<commit_message>
added RFC resolution_by_agencies, which now replaces other RFC/RFR resolution xlxs files for all FY19+ data.  csv code updated to pull pre-FY19 and post-FY19 data from separate files (QC verified the summation across agencies in new file produced identical CSVs)
</commit_message>
<xml_diff>
--- a/bin/pending_rfcs_source.xlsx
+++ b/bin/pending_rfcs_source.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\IQA\iqa\bin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3066F0E9-51C2-43AC-BA76-F3BCB61E7CB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ADFDD73-E6A9-4058-A6DC-2F045DBDEF4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CD4E6399-B2A4-4637-80A1-F963F6DA3DE5}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Year</t>
   </si>
@@ -84,21 +84,6 @@
     <t>FY18</t>
   </si>
   <si>
-    <t>FY19</t>
-  </si>
-  <si>
-    <t>FY20</t>
-  </si>
-  <si>
-    <t>FY21</t>
-  </si>
-  <si>
-    <t>FY22</t>
-  </si>
-  <si>
-    <t>FY23</t>
-  </si>
-  <si>
     <t>Correction</t>
   </si>
   <si>
@@ -115,12 +100,6 @@
   </si>
   <si>
     <t>FY03-04</t>
-  </si>
-  <si>
-    <t>FY24</t>
-  </si>
-  <si>
-    <t>FY25</t>
   </si>
 </sst>
 </file>
@@ -497,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CD143C0-3FFE-403D-8194-F73A02D5ED39}">
-  <dimension ref="A1:T23"/>
+  <dimension ref="A1:T21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="13" max="13" width="13.42578125" customWidth="1"/>
@@ -510,24 +489,24 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C1" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="F1" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -874,150 +853,20 @@
       </c>
       <c r="G16" s="2"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>15</v>
-      </c>
-      <c r="B17">
-        <v>0</v>
-      </c>
-      <c r="C17">
-        <v>0</v>
-      </c>
-      <c r="D17">
-        <v>0</v>
-      </c>
-      <c r="E17">
-        <v>0</v>
-      </c>
-      <c r="F17">
-        <v>0</v>
-      </c>
+    <row r="17" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G17" s="2"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>16</v>
-      </c>
-      <c r="B18">
-        <v>0</v>
-      </c>
-      <c r="C18">
-        <v>0</v>
-      </c>
-      <c r="D18">
-        <v>0</v>
-      </c>
-      <c r="E18">
-        <v>0</v>
-      </c>
-      <c r="F18">
-        <v>0</v>
-      </c>
+    <row r="18" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G18" s="2"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B19">
-        <v>0</v>
-      </c>
-      <c r="C19">
-        <v>0</v>
-      </c>
-      <c r="D19">
-        <v>0</v>
-      </c>
-      <c r="E19">
-        <v>0</v>
-      </c>
-      <c r="F19">
-        <v>0</v>
-      </c>
+    <row r="19" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G19" s="2"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>18</v>
-      </c>
-      <c r="B20">
-        <v>0</v>
-      </c>
-      <c r="C20">
-        <v>0</v>
-      </c>
-      <c r="D20">
-        <v>0</v>
-      </c>
-      <c r="E20">
-        <v>0</v>
-      </c>
-      <c r="F20">
-        <v>0</v>
-      </c>
+    <row r="20" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G20" s="2"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>19</v>
-      </c>
-      <c r="B21">
-        <v>0</v>
-      </c>
-      <c r="C21">
-        <v>0</v>
-      </c>
-      <c r="D21">
-        <v>0</v>
-      </c>
-      <c r="E21">
-        <v>0</v>
-      </c>
-      <c r="F21">
-        <v>0</v>
-      </c>
+    <row r="21" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G21" s="2"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>26</v>
-      </c>
-      <c r="B22">
-        <v>0</v>
-      </c>
-      <c r="C22">
-        <v>0</v>
-      </c>
-      <c r="D22">
-        <v>0</v>
-      </c>
-      <c r="E22">
-        <v>0</v>
-      </c>
-      <c r="F22">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>27</v>
-      </c>
-      <c r="B23">
-        <v>0</v>
-      </c>
-      <c r="C23">
-        <v>0</v>
-      </c>
-      <c r="D23">
-        <v>0</v>
-      </c>
-      <c r="E23">
-        <v>0</v>
-      </c>
-      <c r="F23">
-        <v>0</v>
-      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>